<commit_message>
data: regenerate snapshots after WM W28 sales edit (local ETL run)
Operator's WM W28 other_channels.xlsx edit added 15 additional 1P units
(200 -> 215, INR 4.13L -> 4.47L).  Ran business_report_derive -> sales_auto_etl
-> business_ads_weekly_etl -> step3 -> step4 -> step5 locally on origin
state so snapshots reflect the edit without waiting for CI (Amazon Ads
still flaky today).

Verified end-to-end:
- weekly_sales_snapshot.csv: W28 WM 1p Sales 215 units / INR 4.47L
- business_ads_joined.csv: 3404 rows, 4419 dropped, clean
- AMS Trend last-12w ex-Fossil: INR 8.23 Cr / TACOS 12.78%
- Brand-mistag gate: clean (0 definite mistags)

step4 notna() fix (1ec0182) still holds; no phantom AA rows in output.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ams_weekly_data/White_Mulberry/business_report_week28.xlsx
+++ b/data/ams_weekly_data/White_Mulberry/business_report_week28.xlsx
@@ -1088,7 +1088,7 @@
         <v>0</v>
       </c>
       <c r="P8" t="n">
-        <v>17</v>
+        <v>96</v>
       </c>
       <c r="Q8" t="n">
         <v>0</v>
@@ -1100,7 +1100,7 @@
         <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>39519.49</v>
+        <v>214558.24</v>
       </c>
       <c r="U8" t="n">
         <v>0</v>
@@ -1169,7 +1169,7 @@
         <v>0</v>
       </c>
       <c r="P9" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="Q9" t="n">
         <v>0</v>
@@ -1181,7 +1181,7 @@
         <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>29823.73</v>
+        <v>54457.64</v>
       </c>
       <c r="U9" t="n">
         <v>0</v>
@@ -1250,7 +1250,7 @@
         <v>0</v>
       </c>
       <c r="P10" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="Q10" t="n">
         <v>0</v>
@@ -1262,7 +1262,7 @@
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>4444.07</v>
+        <v>8551.700000000001</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
@@ -1331,7 +1331,7 @@
         <v>0</v>
       </c>
       <c r="P11" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="Q11" t="n">
         <v>0</v>
@@ -1343,7 +1343,7 @@
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>2783.9</v>
+        <v>46256.15</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
@@ -1412,7 +1412,7 @@
         <v>0</v>
       </c>
       <c r="P12" t="n">
-        <v>1</v>
+        <v>68</v>
       </c>
       <c r="Q12" t="n">
         <v>0</v>
@@ -1424,7 +1424,7 @@
         <v>0</v>
       </c>
       <c r="T12" t="n">
-        <v>1694.07</v>
+        <v>112493.38</v>
       </c>
       <c r="U12" t="n">
         <v>0</v>
@@ -1736,7 +1736,7 @@
         <v>0</v>
       </c>
       <c r="P16" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="Q16" t="n">
         <v>0</v>
@@ -1748,7 +1748,7 @@
         <v>0</v>
       </c>
       <c r="T16" t="n">
-        <v>3143.22</v>
+        <v>29830.51</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
@@ -1817,7 +1817,7 @@
         <v>0</v>
       </c>
       <c r="P17" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="Q17" t="n">
         <v>0</v>
@@ -1829,7 +1829,7 @@
         <v>0</v>
       </c>
       <c r="T17" t="n">
-        <v>2592.37</v>
+        <v>65186.34</v>
       </c>
       <c r="U17" t="n">
         <v>0</v>

</xml_diff>